<commit_message>
Remove inflation assumption from workbook and sources
</commit_message>
<xml_diff>
--- a/financial-model/output/Engineering_Economy_Analysis.xlsx
+++ b/financial-model/output/Engineering_Economy_Analysis.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="401">
   <si>
     <t>SOURCES &amp; REFERENCES</t>
   </si>
@@ -520,15 +520,6 @@
   </si>
   <si>
     <t>Project proposal</t>
-  </si>
-  <si>
-    <t>General Inflation (informational)</t>
-  </si>
-  <si>
-    <t>Analysis conducted in constant real dollars; MARR already includes a market risk premium.</t>
-  </si>
-  <si>
-    <t>BLS CPI</t>
   </si>
   <si>
     <t>Tax Regime</t>
@@ -3638,7 +3629,7 @@
   <sheetData>
     <row r="2" spans="2:10">
       <c r="B2" s="1" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3649,38 +3640,38 @@
     </row>
     <row r="3" spans="2:10">
       <c r="B3" s="2" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
     </row>
     <row r="5" spans="2:10">
       <c r="B5" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>248</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>251</v>
-      </c>
       <c r="J5" s="17" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="6" spans="2:10">
       <c r="B6" s="4" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="C6" s="18">
         <v>-15000</v>
@@ -3707,7 +3698,7 @@
     </row>
     <row r="7" spans="2:10">
       <c r="B7" s="4" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="C7" s="18">
         <v>-370000</v>
@@ -3734,7 +3725,7 @@
     </row>
     <row r="9" spans="2:10">
       <c r="B9" s="3" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -3747,24 +3738,24 @@
     </row>
     <row r="10" spans="2:10">
       <c r="B10" s="6" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D10" s="17" t="s">
         <v>111</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
     </row>
     <row r="11" spans="2:10">
       <c r="B11" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C11" s="24">
         <f>J6</f>
@@ -3785,7 +3776,7 @@
     </row>
     <row r="12" spans="2:10">
       <c r="B12" s="4" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C12" s="24">
         <f>J7</f>
@@ -3806,7 +3797,7 @@
     </row>
     <row r="14" spans="2:10">
       <c r="B14" s="10" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
@@ -3852,7 +3843,7 @@
   <sheetData>
     <row r="2" spans="2:7">
       <c r="B2" s="1" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3862,29 +3853,29 @@
     </row>
     <row r="3" spans="2:7">
       <c r="B3" s="2" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
     </row>
     <row r="5" spans="2:7">
       <c r="B5" s="6" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="2:7">
       <c r="B6" s="4" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="C6" s="20">
         <v>15000</v>
@@ -3896,12 +3887,12 @@
         <v>355000</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
     </row>
     <row r="7" spans="2:7">
       <c r="B7" s="4" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C7" s="20">
         <v>179000</v>
@@ -3913,12 +3904,12 @@
         <v>151000</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
     </row>
     <row r="8" spans="2:7">
       <c r="B8" s="5" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C8" s="18">
         <v>0</v>
@@ -3932,7 +3923,7 @@
     </row>
     <row r="9" spans="2:7">
       <c r="B9" s="4" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="C9" s="20">
         <v>600035.7625440408</v>
@@ -3950,7 +3941,7 @@
     </row>
     <row r="10" spans="2:7">
       <c r="B10" s="4" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="C10" s="20">
         <v>15000</v>
@@ -3964,7 +3955,7 @@
     </row>
     <row r="11" spans="2:7">
       <c r="B11" s="4" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="C11" s="23">
         <v>40.00238416960272</v>
@@ -3982,7 +3973,7 @@
     </row>
     <row r="12" spans="2:7">
       <c r="B12" s="5" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="C12" s="21">
         <v>40.00238416960272</v>
@@ -3994,26 +3985,26 @@
         <v>1.537886080629816</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="13" spans="2:7">
       <c r="B13" s="4" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="E13" s="26" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="15" spans="2:7">
       <c r="B15" s="10" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
@@ -4065,7 +4056,7 @@
   <sheetData>
     <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -4074,12 +4065,12 @@
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="2" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="5" spans="2:6">
       <c r="B5" s="3" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -4088,12 +4079,12 @@
     </row>
     <row r="6" spans="2:6">
       <c r="B6" s="12" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="7" spans="2:6">
       <c r="B7" s="4" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="C7" s="20">
         <v>165000</v>
@@ -4101,7 +4092,7 @@
     </row>
     <row r="8" spans="2:6">
       <c r="B8" s="4" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="C8" s="20">
         <v>225000</v>
@@ -4109,7 +4100,7 @@
     </row>
     <row r="9" spans="2:6">
       <c r="B9" s="4" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="C9" s="20">
         <v>326494.6657384585</v>
@@ -4117,24 +4108,24 @@
     </row>
     <row r="10" spans="2:6">
       <c r="B10" s="4" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="C10" s="22">
         <v>52837.17007128108</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
     </row>
     <row r="11" spans="2:6">
       <c r="B11" s="4" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
@@ -4142,7 +4133,7 @@
     </row>
     <row r="13" spans="2:6">
       <c r="B13" s="3" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
@@ -4151,18 +4142,18 @@
     </row>
     <row r="14" spans="2:6">
       <c r="B14" s="4" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="C14" s="18">
         <v>50000</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
     </row>
     <row r="15" spans="2:6">
       <c r="B15" s="4" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="C15" s="18">
         <v>480000</v>
@@ -4170,21 +4161,21 @@
     </row>
     <row r="16" spans="2:6">
       <c r="B16" s="4" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="C16" s="23">
         <v>-3.129769795723135</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
     </row>
     <row r="17" spans="2:6">
       <c r="B17" s="4" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
@@ -4192,7 +4183,7 @@
     </row>
     <row r="19" spans="2:6">
       <c r="B19" s="3" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -4201,23 +4192,23 @@
     </row>
     <row r="20" spans="2:6">
       <c r="B20" s="12" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
     </row>
     <row r="21" spans="2:6">
       <c r="B21" s="4" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="C21" s="24">
         <v>0.8602001226515239</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
     </row>
     <row r="22" spans="2:6">
       <c r="B22" s="5" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="C22" s="25">
         <f>MARR</f>
@@ -4226,21 +4217,21 @@
     </row>
     <row r="23" spans="2:6">
       <c r="B23" s="4" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="C23" s="24">
         <f>C21-C22</f>
         <v>0</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
     </row>
     <row r="25" spans="2:6">
       <c r="B25" s="3" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
@@ -4249,30 +4240,30 @@
     </row>
     <row r="26" spans="2:6">
       <c r="B26" s="12" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
     </row>
     <row r="27" spans="2:6">
       <c r="B27" s="4" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="C27" s="22">
         <v>-47872122.44653919</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
     </row>
     <row r="28" spans="2:6">
       <c r="B28" s="5" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="C28" s="18">
         <f>ACTIVE_VALUE</f>
         <v>0</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
@@ -4312,7 +4303,7 @@
   <sheetData>
     <row r="2" spans="2:8">
       <c r="B2" s="1" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -4323,29 +4314,29 @@
     </row>
     <row r="3" spans="2:8">
       <c r="B3" s="2" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
     </row>
     <row r="5" spans="2:8">
       <c r="B5" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>361</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>362</v>
+      </c>
+      <c r="E5" s="17" t="s">
         <v>363</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="F5" s="17" t="s">
         <v>364</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>365</v>
-      </c>
-      <c r="E5" s="17" t="s">
-        <v>366</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="6" spans="2:8">
       <c r="B6" s="4" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="C6" s="18">
         <v>-943613.7788181889</v>
@@ -4362,7 +4353,7 @@
     </row>
     <row r="7" spans="2:8">
       <c r="B7" s="4" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="C7" s="18">
         <v>-1183253.317272169</v>
@@ -4379,7 +4370,7 @@
     </row>
     <row r="8" spans="2:8">
       <c r="B8" s="4" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="C8" s="18">
         <v>-1018460.758228702</v>
@@ -4396,7 +4387,7 @@
     </row>
     <row r="9" spans="2:8">
       <c r="B9" s="4" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="C9" s="18">
         <v>-1069319.594993616</v>
@@ -4413,7 +4404,7 @@
     </row>
     <row r="10" spans="2:8">
       <c r="B10" s="4" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C10" s="18">
         <v>-1114347.827640634</v>
@@ -4430,7 +4421,7 @@
     </row>
     <row r="11" spans="2:8">
       <c r="B11" s="15" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="C11" s="15"/>
       <c r="D11" s="15"/>
@@ -4439,18 +4430,18 @@
     </row>
     <row r="12" spans="2:8">
       <c r="B12" s="6" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="13" spans="2:8">
       <c r="B13" s="5" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="C13" s="18">
         <v>150846.9794105131</v>
@@ -4461,7 +4452,7 @@
     </row>
     <row r="14" spans="2:8">
       <c r="B14" s="5" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="C14" s="18">
         <v>-88792.55904346704</v>
@@ -4472,7 +4463,7 @@
     </row>
     <row r="15" spans="2:8">
       <c r="B15" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="C15" s="18">
         <v>76000.00000000012</v>
@@ -4483,7 +4474,7 @@
     </row>
     <row r="16" spans="2:8">
       <c r="B16" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="C16" s="18">
         <v>25141.16323508555</v>
@@ -4494,7 +4485,7 @@
     </row>
     <row r="17" spans="2:4">
       <c r="B17" s="5" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C17" s="18">
         <v>-19887.06941193156</v>
@@ -4505,7 +4496,7 @@
     </row>
     <row r="40" spans="2:6">
       <c r="B40" s="3" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
@@ -4514,24 +4505,24 @@
     </row>
     <row r="41" spans="2:6">
       <c r="B41" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="C41" s="17" t="s">
+        <v>375</v>
+      </c>
+      <c r="D41" s="17" t="s">
+        <v>376</v>
+      </c>
+      <c r="E41" s="17" t="s">
         <v>377</v>
       </c>
-      <c r="C41" s="17" t="s">
+      <c r="F41" s="7" t="s">
         <v>378</v>
-      </c>
-      <c r="D41" s="17" t="s">
-        <v>379</v>
-      </c>
-      <c r="E41" s="17" t="s">
-        <v>380</v>
-      </c>
-      <c r="F41" s="7" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="42" spans="2:6">
       <c r="B42" s="4" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="C42" s="18">
         <v>-2242535.295275593</v>
@@ -4543,12 +4534,12 @@
         <v>-1265194.807051147</v>
       </c>
       <c r="F42" s="26" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="43" spans="2:6">
       <c r="B43" s="4" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="C43" s="18">
         <v>-1870446.079396327</v>
@@ -4560,12 +4551,12 @@
         <v>-1094460.758228702</v>
       </c>
       <c r="F43" s="26" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="44" spans="2:6">
       <c r="B44" s="4" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="C44" s="18">
         <v>-1498356.863517062</v>
@@ -4577,7 +4568,7 @@
         <v>-923726.7094062574</v>
       </c>
       <c r="F44" s="26" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
   </sheetData>
@@ -4607,7 +4598,7 @@
   <sheetData>
     <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -4616,12 +4607,12 @@
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="2" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="5" spans="2:6">
       <c r="B5" s="27" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="C5" s="27"/>
       <c r="D5" s="27"/>
@@ -4637,7 +4628,7 @@
     </row>
     <row r="9" spans="2:6">
       <c r="B9" s="3" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -4646,24 +4637,24 @@
     </row>
     <row r="10" spans="2:6">
       <c r="B10" s="6" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="11" spans="2:6">
       <c r="B11" s="4" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C11" s="18">
         <v>10000</v>
@@ -4678,7 +4669,7 @@
     </row>
     <row r="12" spans="2:6">
       <c r="B12" s="4" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C12" s="18">
         <v>555000</v>
@@ -4693,7 +4684,7 @@
     </row>
     <row r="13" spans="2:6">
       <c r="B13" s="4" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="C13" s="18">
         <v>0</v>
@@ -4708,7 +4699,7 @@
     </row>
     <row r="14" spans="2:6">
       <c r="B14" s="4" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="C14" s="20">
         <v>-1870446.079396327</v>
@@ -4723,7 +4714,7 @@
     </row>
     <row r="15" spans="2:6">
       <c r="B15" s="4" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="C15" s="20">
         <v>-557983.1555246152</v>
@@ -4738,7 +4729,7 @@
     </row>
     <row r="16" spans="2:6">
       <c r="B16" s="4" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="C16" s="20">
         <v>-3762135.165624998</v>
@@ -4753,7 +4744,7 @@
     </row>
     <row r="18" spans="2:6">
       <c r="B18" s="3" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
@@ -4762,59 +4753,59 @@
     </row>
     <row r="19" spans="2:6">
       <c r="B19" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C19" s="23">
         <v>1.121212121212121</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
     </row>
     <row r="20" spans="2:6">
       <c r="B20" s="4" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="C20" s="24">
         <v>0.8602001226515239</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
     </row>
     <row r="21" spans="2:6">
       <c r="B21" s="4" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="C21" s="23">
         <v>3.097257624777366</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
     </row>
     <row r="22" spans="2:6">
       <c r="B22" s="4" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="C22" s="20">
         <v>330000</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="E22" s="5"/>
       <c r="F22" s="5"/>
     </row>
     <row r="24" spans="2:6">
       <c r="B24" s="3" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
@@ -4823,7 +4814,7 @@
     </row>
     <row r="25" spans="2:6">
       <c r="B25" s="10" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
@@ -5382,13 +5373,11 @@
       <c r="B7" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="C7" s="11">
-        <v>0.025</v>
-      </c>
-      <c r="D7" s="12" t="s">
+      <c r="C7" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="D7" s="5"/>
+      <c r="E7" s="12" t="s">
         <v>164</v>
       </c>
     </row>
@@ -5404,21 +5393,9 @@
         <v>167</v>
       </c>
     </row>
-    <row r="9" spans="2:5">
-      <c r="B9" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="12" t="s">
-        <v>170</v>
-      </c>
-    </row>
     <row r="11" spans="2:5">
       <c r="B11" s="15" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C11" s="15"/>
       <c r="D11" s="15"/>
@@ -5432,24 +5409,24 @@
         <v>50000000</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="2:5">
       <c r="B13" s="4" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="C13" s="16">
         <v>10000000</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="14" spans="2:5">
@@ -5461,38 +5438,38 @@
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="12" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="15" spans="2:5">
       <c r="B15" s="4" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="12" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="16" spans="2:5">
       <c r="B16" s="4" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C16" s="14">
         <v>180</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="18" spans="2:5">
       <c r="B18" s="15" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
@@ -5500,21 +5477,21 @@
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="E19" s="17" t="s">
         <v>184</v>
-      </c>
-      <c r="C19" s="17" t="s">
-        <v>185</v>
-      </c>
-      <c r="D19" s="17" t="s">
-        <v>186</v>
-      </c>
-      <c r="E19" s="17" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" s="4" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C20" s="18">
         <v>10000</v>
@@ -5528,7 +5505,7 @@
     </row>
     <row r="21" spans="2:5">
       <c r="B21" s="4" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C21" s="18">
         <v>25000</v>
@@ -5542,7 +5519,7 @@
     </row>
     <row r="22" spans="2:5">
       <c r="B22" s="4" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C22" s="18">
         <v>380000</v>
@@ -5557,8 +5534,8 @@
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="B2:E2"/>
+    <mergeCell ref="C7:D7"/>
     <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
     <mergeCell ref="B11:E11"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="C15:D15"/>
@@ -5566,9 +5543,8 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E5" r:id="rId1"/>
-    <hyperlink ref="E7" r:id="rId2"/>
-    <hyperlink ref="E12" r:id="rId3"/>
-    <hyperlink ref="E16" r:id="rId4"/>
+    <hyperlink ref="E12" r:id="rId2"/>
+    <hyperlink ref="E16" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5592,7 +5568,7 @@
   <sheetData>
     <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -5601,12 +5577,12 @@
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="2" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" spans="2:6">
       <c r="B6" s="3" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -5618,16 +5594,16 @@
         <v>2</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" spans="2:6">
@@ -5635,13 +5611,13 @@
         <v>1</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D8" s="16">
         <v>10000</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="F8" s="13" t="s">
         <v>42</v>
@@ -5650,7 +5626,7 @@
     <row r="9" spans="2:6">
       <c r="B9" s="5"/>
       <c r="C9" s="4" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D9" s="19">
         <f>SUM(D8:D8)</f>
@@ -5661,7 +5637,7 @@
     </row>
     <row r="11" spans="2:6">
       <c r="B11" s="3" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -5673,16 +5649,16 @@
         <v>2</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="13" spans="2:6">
@@ -5690,13 +5666,13 @@
         <v>1</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D13" s="16">
         <v>25000</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>47</v>
@@ -5705,7 +5681,7 @@
     <row r="14" spans="2:6">
       <c r="B14" s="5"/>
       <c r="C14" s="4" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D14" s="19">
         <f>SUM(D13:D13)</f>
@@ -5716,7 +5692,7 @@
     </row>
     <row r="16" spans="2:6">
       <c r="B16" s="3" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
@@ -5728,16 +5704,16 @@
         <v>2</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="18" spans="2:6">
@@ -5745,13 +5721,13 @@
         <v>1</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D18" s="16">
         <v>60000</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="F18" s="13" t="s">
         <v>72</v>
@@ -5762,13 +5738,13 @@
         <v>2</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D19" s="16">
         <v>20000</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>67</v>
@@ -5779,13 +5755,13 @@
         <v>3</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D20" s="16">
         <v>30000</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F20" s="13" t="s">
         <v>67</v>
@@ -5796,13 +5772,13 @@
         <v>4</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="D21" s="16">
         <v>40000</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F21" s="13" t="s">
         <v>42</v>
@@ -5813,13 +5789,13 @@
         <v>5</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="D22" s="16">
         <v>180000</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="F22" s="13" t="s">
         <v>82</v>
@@ -5830,13 +5806,13 @@
         <v>6</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D23" s="16">
         <v>50000</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="F23" s="13" t="s">
         <v>92</v>
@@ -5845,7 +5821,7 @@
     <row r="24" spans="2:6">
       <c r="B24" s="5"/>
       <c r="C24" s="4" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D24" s="19">
         <f>SUM(D18:D23)</f>
@@ -5893,7 +5869,7 @@
   <sheetData>
     <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -5902,12 +5878,12 @@
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" spans="2:6">
       <c r="B6" s="3" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -5919,16 +5895,16 @@
         <v>2</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" spans="2:6">
@@ -5936,13 +5912,13 @@
         <v>1</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D8" s="16">
         <v>390000</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="F8" s="13" t="s">
         <v>9</v>
@@ -5953,13 +5929,13 @@
         <v>2</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D9" s="16">
         <v>75000</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="F9" s="13" t="s">
         <v>22</v>
@@ -5970,13 +5946,13 @@
         <v>3</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D10" s="16">
         <v>50000</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="F10" s="13" t="s">
         <v>37</v>
@@ -5987,13 +5963,13 @@
         <v>4</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D11" s="16">
         <v>40000</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="F11" s="13" t="s">
         <v>92</v>
@@ -6002,7 +5978,7 @@
     <row r="12" spans="2:6">
       <c r="B12" s="5"/>
       <c r="C12" s="4" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D12" s="19">
         <f>SUM(D8:D11)</f>
@@ -6013,7 +5989,7 @@
     </row>
     <row r="14" spans="2:6">
       <c r="B14" s="3" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
@@ -6025,16 +6001,16 @@
         <v>2</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="16" spans="2:6">
@@ -6042,13 +6018,13 @@
         <v>1</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D16" s="16">
         <v>180000</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="F16" s="13" t="s">
         <v>47</v>
@@ -6059,13 +6035,13 @@
         <v>2</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D17" s="16">
         <v>36000</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="F17" s="13" t="s">
         <v>52</v>
@@ -6076,13 +6052,13 @@
         <v>3</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D18" s="16">
         <v>130000</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="F18" s="13" t="s">
         <v>9</v>
@@ -6093,13 +6069,13 @@
         <v>4</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D19" s="16">
         <v>20000</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>57</v>
@@ -6110,13 +6086,13 @@
         <v>5</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D20" s="16">
         <v>10000</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="F20" s="13" t="s">
         <v>37</v>
@@ -6125,7 +6101,7 @@
     <row r="21" spans="2:6">
       <c r="B21" s="5"/>
       <c r="C21" s="4" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D21" s="19">
         <f>SUM(D16:D20)</f>
@@ -6136,7 +6112,7 @@
     </row>
     <row r="23" spans="2:6">
       <c r="B23" s="3" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
@@ -6148,16 +6124,16 @@
         <v>2</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="25" spans="2:6">
@@ -6165,13 +6141,13 @@
         <v>1</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D25" s="16">
         <v>145000</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>82</v>
@@ -6182,13 +6158,13 @@
         <v>2</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D26" s="16">
         <v>30000</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="F26" s="13" t="s">
         <v>77</v>
@@ -6199,13 +6175,13 @@
         <v>3</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D27" s="16">
         <v>25000</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="F27" s="13" t="s">
         <v>72</v>
@@ -6216,13 +6192,13 @@
         <v>4</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D28" s="16">
         <v>15000</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="F28" s="13" t="s">
         <v>57</v>
@@ -6233,13 +6209,13 @@
         <v>5</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D29" s="16">
         <v>10000</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="F29" s="13" t="s">
         <v>37</v>
@@ -6248,7 +6224,7 @@
     <row r="30" spans="2:6">
       <c r="B30" s="5"/>
       <c r="C30" s="4" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D30" s="19">
         <f>SUM(D25:D29)</f>
@@ -6300,7 +6276,7 @@
   <sheetData>
     <row r="2" spans="2:10">
       <c r="B2" s="1" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -6312,35 +6288,35 @@
     </row>
     <row r="3" spans="2:10">
       <c r="B3" s="2" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="5" spans="2:10">
       <c r="B5" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>248</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="6" spans="2:10">
       <c r="B6" s="4" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C6" s="18">
         <v>-10000</v>
@@ -6361,15 +6337,15 @@
         <v>0</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
     <row r="7" spans="2:10">
       <c r="B7" s="5" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C7" s="18">
         <v>0</v>
@@ -6390,7 +6366,7 @@
         <v>-390000</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="J7" s="18">
         <v>-10000</v>
@@ -6398,7 +6374,7 @@
     </row>
     <row r="8" spans="2:10">
       <c r="B8" s="5" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C8" s="18">
         <v>0</v>
@@ -6419,7 +6395,7 @@
         <v>-75000</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="J8" s="18">
         <v>-555000</v>
@@ -6427,7 +6403,7 @@
     </row>
     <row r="9" spans="2:10">
       <c r="B9" s="5" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C9" s="18">
         <v>0</v>
@@ -6448,7 +6424,7 @@
         <v>-50000</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="J9" s="18">
         <v>0</v>
@@ -6456,7 +6432,7 @@
     </row>
     <row r="10" spans="2:10">
       <c r="B10" s="5" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C10" s="18">
         <v>0</v>
@@ -6477,7 +6453,7 @@
         <v>-40000</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="J10" s="20">
         <f>H15</f>
@@ -6486,7 +6462,7 @@
     </row>
     <row r="11" spans="2:10">
       <c r="B11" s="4" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="C11" s="20">
         <f>SUM(C6:C10)</f>
@@ -6515,7 +6491,7 @@
     </row>
     <row r="12" spans="2:10">
       <c r="B12" s="5" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C12" s="21">
         <f>1/(1+MARR)^0</f>
@@ -6544,7 +6520,7 @@
     </row>
     <row r="13" spans="2:10">
       <c r="B13" s="4" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C13" s="20">
         <f>C11*C12</f>
@@ -6573,7 +6549,7 @@
     </row>
     <row r="14" spans="2:10">
       <c r="B14" s="4" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C14" s="20">
         <f>C11</f>
@@ -6602,7 +6578,7 @@
     </row>
     <row r="15" spans="2:10">
       <c r="B15" s="4" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C15" s="20">
         <f>C13</f>
@@ -6654,7 +6630,7 @@
   <sheetData>
     <row r="2" spans="2:10">
       <c r="B2" s="1" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -6666,35 +6642,35 @@
     </row>
     <row r="3" spans="2:10">
       <c r="B3" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" spans="2:10">
       <c r="B5" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>248</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="6" spans="2:10">
       <c r="B6" s="4" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C6" s="18">
         <v>-25000</v>
@@ -6715,15 +6691,15 @@
         <v>0</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
     <row r="7" spans="2:10">
       <c r="B7" s="5" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C7" s="18">
         <v>0</v>
@@ -6744,7 +6720,7 @@
         <v>-180000</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="J7" s="18">
         <v>-25000</v>
@@ -6752,7 +6728,7 @@
     </row>
     <row r="8" spans="2:10">
       <c r="B8" s="5" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C8" s="18">
         <v>0</v>
@@ -6773,7 +6749,7 @@
         <v>-36000</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="J8" s="18">
         <v>-376000</v>
@@ -6781,7 +6757,7 @@
     </row>
     <row r="9" spans="2:10">
       <c r="B9" s="5" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C9" s="18">
         <v>0</v>
@@ -6802,7 +6778,7 @@
         <v>-130000</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="J9" s="18">
         <v>0</v>
@@ -6810,7 +6786,7 @@
     </row>
     <row r="10" spans="2:10">
       <c r="B10" s="5" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C10" s="18">
         <v>0</v>
@@ -6831,7 +6807,7 @@
         <v>-20000</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="J10" s="20">
         <f>H16</f>
@@ -6840,7 +6816,7 @@
     </row>
     <row r="11" spans="2:10">
       <c r="B11" s="5" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C11" s="18">
         <v>0</v>
@@ -6863,7 +6839,7 @@
     </row>
     <row r="12" spans="2:10">
       <c r="B12" s="4" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="C12" s="20">
         <f>SUM(C6:C11)</f>
@@ -6892,7 +6868,7 @@
     </row>
     <row r="13" spans="2:10">
       <c r="B13" s="5" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C13" s="21">
         <f>1/(1+MARR)^0</f>
@@ -6921,7 +6897,7 @@
     </row>
     <row r="14" spans="2:10">
       <c r="B14" s="4" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C14" s="20">
         <f>C12*C13</f>
@@ -6950,7 +6926,7 @@
     </row>
     <row r="15" spans="2:10">
       <c r="B15" s="4" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C15" s="20">
         <f>C12</f>
@@ -6979,7 +6955,7 @@
     </row>
     <row r="16" spans="2:10">
       <c r="B16" s="4" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C16" s="20">
         <f>C14</f>
@@ -7031,7 +7007,7 @@
   <sheetData>
     <row r="2" spans="2:10">
       <c r="B2" s="1" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -7043,35 +7019,35 @@
     </row>
     <row r="3" spans="2:10">
       <c r="B3" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" spans="2:10">
       <c r="B5" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>248</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="6" spans="2:10">
       <c r="B6" s="4" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C6" s="18">
         <v>-380000</v>
@@ -7092,15 +7068,15 @@
         <v>0</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
     <row r="7" spans="2:10">
       <c r="B7" s="5" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C7" s="18">
         <v>0</v>
@@ -7121,7 +7097,7 @@
         <v>-145000</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="J7" s="18">
         <v>-380000</v>
@@ -7129,7 +7105,7 @@
     </row>
     <row r="8" spans="2:10">
       <c r="B8" s="5" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C8" s="18">
         <v>0</v>
@@ -7150,7 +7126,7 @@
         <v>-30000</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="J8" s="18">
         <v>-225000</v>
@@ -7158,7 +7134,7 @@
     </row>
     <row r="9" spans="2:10">
       <c r="B9" s="5" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C9" s="18">
         <v>0</v>
@@ -7179,7 +7155,7 @@
         <v>-25000</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="J9" s="18">
         <v>80000</v>
@@ -7187,7 +7163,7 @@
     </row>
     <row r="10" spans="2:10">
       <c r="B10" s="5" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C10" s="18">
         <v>0</v>
@@ -7208,7 +7184,7 @@
         <v>-15000</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="J10" s="22">
         <f>H17</f>
@@ -7217,7 +7193,7 @@
     </row>
     <row r="11" spans="2:10">
       <c r="B11" s="5" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C11" s="18">
         <v>0</v>
@@ -7240,7 +7216,7 @@
     </row>
     <row r="12" spans="2:10">
       <c r="B12" s="4" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C12" s="18">
         <v>0</v>
@@ -7263,7 +7239,7 @@
     </row>
     <row r="13" spans="2:10">
       <c r="B13" s="4" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="C13" s="20">
         <f>SUM(C6:C12)</f>
@@ -7292,7 +7268,7 @@
     </row>
     <row r="14" spans="2:10">
       <c r="B14" s="5" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C14" s="21">
         <f>1/(1+MARR)^0</f>
@@ -7321,7 +7297,7 @@
     </row>
     <row r="15" spans="2:10">
       <c r="B15" s="4" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C15" s="20">
         <f>C13*C14</f>
@@ -7350,7 +7326,7 @@
     </row>
     <row r="16" spans="2:10">
       <c r="B16" s="4" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C16" s="20">
         <f>C13</f>
@@ -7379,7 +7355,7 @@
     </row>
     <row r="17" spans="2:8">
       <c r="B17" s="4" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C17" s="20">
         <f>C15</f>
@@ -7431,7 +7407,7 @@
   <sheetData>
     <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -7440,29 +7416,29 @@
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="2" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" spans="2:6">
       <c r="B5" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>266</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>267</v>
+      </c>
+      <c r="E5" s="17" t="s">
         <v>268</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="F5" s="6" t="s">
         <v>269</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>270</v>
-      </c>
-      <c r="E5" s="17" t="s">
-        <v>271</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="6" spans="2:6">
       <c r="B6" s="4" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="C6" s="20">
         <f>'05. CF — Alt 1 Manual'!H15</f>
@@ -7477,12 +7453,12 @@
         <v>0</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="7" spans="2:6">
       <c r="B7" s="4" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C7" s="20">
         <f>C6*MARR*(1+MARR)^STUDY_PERIOD/((1+MARR)^STUDY_PERIOD-1)</f>
@@ -7503,7 +7479,7 @@
     </row>
     <row r="8" spans="2:6">
       <c r="B8" s="4" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="C8" s="20">
         <f>C6*(1+MARR)^STUDY_PERIOD</f>
@@ -7524,7 +7500,7 @@
     </row>
     <row r="10" spans="2:6">
       <c r="B10" s="15" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C10" s="15"/>
       <c r="D10" s="15"/>
@@ -7533,13 +7509,13 @@
     </row>
     <row r="11" spans="2:6">
       <c r="B11" s="5" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="C11" s="21">
         <v>3.352155098011401</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="E11" s="21">
         <v>0.4971767352982899</v>
@@ -7547,13 +7523,13 @@
     </row>
     <row r="12" spans="2:6">
       <c r="B12" s="5" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="C12" s="21">
         <v>0.2983155524615284</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="E12" s="21">
         <v>2.011357187499999</v>
@@ -7584,7 +7560,7 @@
   <sheetData>
     <row r="2" spans="2:9">
       <c r="B2" s="1" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -7595,12 +7571,12 @@
     </row>
     <row r="3" spans="2:9">
       <c r="B3" s="2" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" spans="2:9">
       <c r="B5" s="4" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="C5" s="20">
         <v>555000</v>
@@ -7608,7 +7584,7 @@
     </row>
     <row r="6" spans="2:9">
       <c r="B6" s="4" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C6" s="20">
         <v>10000</v>
@@ -7616,7 +7592,7 @@
     </row>
     <row r="9" spans="2:9">
       <c r="B9" s="3" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -7627,7 +7603,7 @@
     </row>
     <row r="10" spans="2:9">
       <c r="B10" s="4" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C10" s="20">
         <v>15000</v>
@@ -7635,7 +7611,7 @@
     </row>
     <row r="11" spans="2:9">
       <c r="B11" s="4" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C11" s="20">
         <v>179000</v>
@@ -7643,7 +7619,7 @@
     </row>
     <row r="12" spans="2:9">
       <c r="B12" s="5" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="C12" s="18">
         <v>0</v>
@@ -7651,39 +7627,39 @@
     </row>
     <row r="13" spans="2:9">
       <c r="B13" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C13" s="23">
         <f>C10/C11</f>
         <v>0</v>
       </c>
       <c r="D13" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="G13" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="H13" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="I13" s="7" t="s">
         <v>248</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="14" spans="2:9">
       <c r="B14" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
     </row>
     <row r="15" spans="2:9">
       <c r="B15" s="5" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="D15" s="18">
         <f>-C10</f>
@@ -7712,7 +7688,7 @@
     </row>
     <row r="16" spans="2:9">
       <c r="B16" s="4" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="D16" s="20">
         <f>D15</f>
@@ -7741,18 +7717,18 @@
     </row>
     <row r="17" spans="2:9">
       <c r="B17" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C17" s="23">
         <v>0.09636871508379888</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="19" spans="2:9">
       <c r="B19" s="3" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -7763,7 +7739,7 @@
     </row>
     <row r="20" spans="2:9">
       <c r="B20" s="4" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C20" s="20">
         <v>370000</v>
@@ -7771,7 +7747,7 @@
     </row>
     <row r="21" spans="2:9">
       <c r="B21" s="4" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C21" s="20">
         <v>330000</v>
@@ -7779,7 +7755,7 @@
     </row>
     <row r="22" spans="2:9">
       <c r="B22" s="5" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="C22" s="18">
         <v>80000</v>
@@ -7787,39 +7763,39 @@
     </row>
     <row r="23" spans="2:9">
       <c r="B23" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C23" s="23">
         <f>C20/C21</f>
         <v>0</v>
       </c>
       <c r="D23" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="G23" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="H23" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="I23" s="7" t="s">
         <v>248</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="I23" s="7" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="24" spans="2:9">
       <c r="B24" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
     </row>
     <row r="25" spans="2:9">
       <c r="B25" s="5" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="D25" s="18">
         <f>-C20</f>
@@ -7848,7 +7824,7 @@
     </row>
     <row r="26" spans="2:9">
       <c r="B26" s="4" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="D26" s="20">
         <f>D25</f>
@@ -7877,18 +7853,18 @@
     </row>
     <row r="27" spans="2:9">
       <c r="B27" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C27" s="23">
         <v>1.33280303030303</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="30" spans="2:9">
       <c r="B30" s="15" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C30" s="15"/>
       <c r="D30" s="15"/>
@@ -7899,7 +7875,7 @@
     </row>
     <row r="31" spans="2:9">
       <c r="B31" s="6" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C31" s="7">
         <v>0</v>
@@ -7922,7 +7898,7 @@
     </row>
     <row r="32" spans="2:9">
       <c r="B32" s="4" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C32" s="18">
         <v>-15000</v>
@@ -7945,7 +7921,7 @@
     </row>
     <row r="33" spans="2:8">
       <c r="B33" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C33" s="18">
         <v>-370000</v>

</xml_diff>

<commit_message>
Remove tax-regime and depreciation rows from Assumptions
</commit_message>
<xml_diff>
--- a/financial-model/output/Engineering_Economy_Analysis.xlsx
+++ b/financial-model/output/Engineering_Economy_Analysis.xlsx
@@ -24,9 +24,9 @@
     <sheet name="15. Sources" sheetId="15" r:id="rId15"/>
   </sheets>
   <definedNames>
-    <definedName name="ACTIVE_VALUE">'02. Assumptions'!$C$13</definedName>
+    <definedName name="ACTIVE_VALUE">'02. Assumptions'!$C$10</definedName>
     <definedName name="MARR">'02. Assumptions'!$C$5</definedName>
-    <definedName name="PROJECT_VALUE">'02. Assumptions'!$C$12</definedName>
+    <definedName name="PROJECT_VALUE">'02. Assumptions'!$C$9</definedName>
     <definedName name="STUDY_PERIOD">'02. Assumptions'!$C$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="395">
   <si>
     <t>SOURCES &amp; REFERENCES</t>
   </si>
@@ -520,24 +520,6 @@
   </si>
   <si>
     <t>Project proposal</t>
-  </si>
-  <si>
-    <t>Tax Regime</t>
-  </si>
-  <si>
-    <t>Pre-tax (course convention)</t>
-  </si>
-  <si>
-    <t>Course convention</t>
-  </si>
-  <si>
-    <t>Depreciation</t>
-  </si>
-  <si>
-    <t>Straight-line, n=5</t>
-  </si>
-  <si>
-    <t>Straight-line for simplicity</t>
   </si>
   <si>
     <t>PROJECT CONTEXT</t>
@@ -3629,7 +3611,7 @@
   <sheetData>
     <row r="2" spans="2:10">
       <c r="B2" s="1" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3640,38 +3622,38 @@
     </row>
     <row r="3" spans="2:10">
       <c r="B3" s="2" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
     </row>
     <row r="5" spans="2:10">
       <c r="B5" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="C5" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>246</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>248</v>
-      </c>
       <c r="J5" s="17" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
     </row>
     <row r="6" spans="2:10">
       <c r="B6" s="4" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="C6" s="18">
         <v>-15000</v>
@@ -3698,7 +3680,7 @@
     </row>
     <row r="7" spans="2:10">
       <c r="B7" s="4" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="C7" s="18">
         <v>-370000</v>
@@ -3725,7 +3707,7 @@
     </row>
     <row r="9" spans="2:10">
       <c r="B9" s="3" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -3738,24 +3720,24 @@
     </row>
     <row r="10" spans="2:10">
       <c r="B10" s="6" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="D10" s="17" t="s">
         <v>111</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
     </row>
     <row r="11" spans="2:10">
       <c r="B11" s="4" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="C11" s="24">
         <f>J6</f>
@@ -3776,7 +3758,7 @@
     </row>
     <row r="12" spans="2:10">
       <c r="B12" s="4" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="C12" s="24">
         <f>J7</f>
@@ -3797,7 +3779,7 @@
     </row>
     <row r="14" spans="2:10">
       <c r="B14" s="10" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
@@ -3843,7 +3825,7 @@
   <sheetData>
     <row r="2" spans="2:7">
       <c r="B2" s="1" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3853,29 +3835,29 @@
     </row>
     <row r="3" spans="2:7">
       <c r="B3" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
     </row>
     <row r="5" spans="2:7">
       <c r="B5" s="6" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6" spans="2:7">
       <c r="B6" s="4" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="C6" s="20">
         <v>15000</v>
@@ -3887,12 +3869,12 @@
         <v>355000</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
     </row>
     <row r="7" spans="2:7">
       <c r="B7" s="4" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="C7" s="20">
         <v>179000</v>
@@ -3904,12 +3886,12 @@
         <v>151000</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
     </row>
     <row r="8" spans="2:7">
       <c r="B8" s="5" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="C8" s="18">
         <v>0</v>
@@ -3923,7 +3905,7 @@
     </row>
     <row r="9" spans="2:7">
       <c r="B9" s="4" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="C9" s="20">
         <v>600035.7625440408</v>
@@ -3941,7 +3923,7 @@
     </row>
     <row r="10" spans="2:7">
       <c r="B10" s="4" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="C10" s="20">
         <v>15000</v>
@@ -3955,7 +3937,7 @@
     </row>
     <row r="11" spans="2:7">
       <c r="B11" s="4" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="C11" s="23">
         <v>40.00238416960272</v>
@@ -3973,7 +3955,7 @@
     </row>
     <row r="12" spans="2:7">
       <c r="B12" s="5" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="C12" s="21">
         <v>40.00238416960272</v>
@@ -3985,26 +3967,26 @@
         <v>1.537886080629816</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
     </row>
     <row r="13" spans="2:7">
       <c r="B13" s="4" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="E13" s="26" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
     </row>
     <row r="15" spans="2:7">
       <c r="B15" s="10" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
@@ -4056,7 +4038,7 @@
   <sheetData>
     <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -4065,12 +4047,12 @@
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="2" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
     </row>
     <row r="5" spans="2:6">
       <c r="B5" s="3" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -4079,12 +4061,12 @@
     </row>
     <row r="6" spans="2:6">
       <c r="B6" s="12" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
     </row>
     <row r="7" spans="2:6">
       <c r="B7" s="4" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="C7" s="20">
         <v>165000</v>
@@ -4092,7 +4074,7 @@
     </row>
     <row r="8" spans="2:6">
       <c r="B8" s="4" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="C8" s="20">
         <v>225000</v>
@@ -4100,7 +4082,7 @@
     </row>
     <row r="9" spans="2:6">
       <c r="B9" s="4" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="C9" s="20">
         <v>326494.6657384585</v>
@@ -4108,24 +4090,24 @@
     </row>
     <row r="10" spans="2:6">
       <c r="B10" s="4" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="C10" s="22">
         <v>52837.17007128108</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
     </row>
     <row r="11" spans="2:6">
       <c r="B11" s="4" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
@@ -4133,7 +4115,7 @@
     </row>
     <row r="13" spans="2:6">
       <c r="B13" s="3" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
@@ -4142,18 +4124,18 @@
     </row>
     <row r="14" spans="2:6">
       <c r="B14" s="4" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="C14" s="18">
         <v>50000</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
     </row>
     <row r="15" spans="2:6">
       <c r="B15" s="4" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="C15" s="18">
         <v>480000</v>
@@ -4161,21 +4143,21 @@
     </row>
     <row r="16" spans="2:6">
       <c r="B16" s="4" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="C16" s="23">
         <v>-3.129769795723135</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
     </row>
     <row r="17" spans="2:6">
       <c r="B17" s="4" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
@@ -4183,7 +4165,7 @@
     </row>
     <row r="19" spans="2:6">
       <c r="B19" s="3" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -4192,23 +4174,23 @@
     </row>
     <row r="20" spans="2:6">
       <c r="B20" s="12" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
     </row>
     <row r="21" spans="2:6">
       <c r="B21" s="4" t="s">
-        <v>347</v>
+        <v>341</v>
       </c>
       <c r="C21" s="24">
         <v>0.8602001226515239</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>348</v>
+        <v>342</v>
       </c>
     </row>
     <row r="22" spans="2:6">
       <c r="B22" s="5" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
       <c r="C22" s="25">
         <f>MARR</f>
@@ -4217,21 +4199,21 @@
     </row>
     <row r="23" spans="2:6">
       <c r="B23" s="4" t="s">
-        <v>350</v>
+        <v>344</v>
       </c>
       <c r="C23" s="24">
         <f>C21-C22</f>
         <v>0</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
     </row>
     <row r="25" spans="2:6">
       <c r="B25" s="3" t="s">
-        <v>352</v>
+        <v>346</v>
       </c>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
@@ -4240,30 +4222,30 @@
     </row>
     <row r="26" spans="2:6">
       <c r="B26" s="12" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
     </row>
     <row r="27" spans="2:6">
       <c r="B27" s="4" t="s">
-        <v>354</v>
+        <v>348</v>
       </c>
       <c r="C27" s="22">
         <v>-47872122.44653919</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
     </row>
     <row r="28" spans="2:6">
       <c r="B28" s="5" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="C28" s="18">
         <f>ACTIVE_VALUE</f>
         <v>0</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
@@ -4303,7 +4285,7 @@
   <sheetData>
     <row r="2" spans="2:8">
       <c r="B2" s="1" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -4314,29 +4296,29 @@
     </row>
     <row r="3" spans="2:8">
       <c r="B3" s="2" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
     </row>
     <row r="5" spans="2:8">
       <c r="B5" s="6" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>362</v>
+        <v>356</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>363</v>
+        <v>357</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
     </row>
     <row r="6" spans="2:8">
       <c r="B6" s="4" t="s">
-        <v>365</v>
+        <v>359</v>
       </c>
       <c r="C6" s="18">
         <v>-943613.7788181889</v>
@@ -4353,7 +4335,7 @@
     </row>
     <row r="7" spans="2:8">
       <c r="B7" s="4" t="s">
-        <v>366</v>
+        <v>360</v>
       </c>
       <c r="C7" s="18">
         <v>-1183253.317272169</v>
@@ -4370,7 +4352,7 @@
     </row>
     <row r="8" spans="2:8">
       <c r="B8" s="4" t="s">
-        <v>367</v>
+        <v>361</v>
       </c>
       <c r="C8" s="18">
         <v>-1018460.758228702</v>
@@ -4387,7 +4369,7 @@
     </row>
     <row r="9" spans="2:8">
       <c r="B9" s="4" t="s">
-        <v>368</v>
+        <v>362</v>
       </c>
       <c r="C9" s="18">
         <v>-1069319.594993616</v>
@@ -4404,7 +4386,7 @@
     </row>
     <row r="10" spans="2:8">
       <c r="B10" s="4" t="s">
-        <v>369</v>
+        <v>363</v>
       </c>
       <c r="C10" s="18">
         <v>-1114347.827640634</v>
@@ -4421,7 +4403,7 @@
     </row>
     <row r="11" spans="2:8">
       <c r="B11" s="15" t="s">
-        <v>370</v>
+        <v>364</v>
       </c>
       <c r="C11" s="15"/>
       <c r="D11" s="15"/>
@@ -4430,18 +4412,18 @@
     </row>
     <row r="12" spans="2:8">
       <c r="B12" s="6" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>371</v>
+        <v>365</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>372</v>
+        <v>366</v>
       </c>
     </row>
     <row r="13" spans="2:8">
       <c r="B13" s="5" t="s">
-        <v>365</v>
+        <v>359</v>
       </c>
       <c r="C13" s="18">
         <v>150846.9794105131</v>
@@ -4452,7 +4434,7 @@
     </row>
     <row r="14" spans="2:8">
       <c r="B14" s="5" t="s">
-        <v>366</v>
+        <v>360</v>
       </c>
       <c r="C14" s="18">
         <v>-88792.55904346704</v>
@@ -4463,7 +4445,7 @@
     </row>
     <row r="15" spans="2:8">
       <c r="B15" s="5" t="s">
-        <v>367</v>
+        <v>361</v>
       </c>
       <c r="C15" s="18">
         <v>76000.00000000012</v>
@@ -4474,7 +4456,7 @@
     </row>
     <row r="16" spans="2:8">
       <c r="B16" s="5" t="s">
-        <v>368</v>
+        <v>362</v>
       </c>
       <c r="C16" s="18">
         <v>25141.16323508555</v>
@@ -4485,7 +4467,7 @@
     </row>
     <row r="17" spans="2:4">
       <c r="B17" s="5" t="s">
-        <v>369</v>
+        <v>363</v>
       </c>
       <c r="C17" s="18">
         <v>-19887.06941193156</v>
@@ -4496,7 +4478,7 @@
     </row>
     <row r="40" spans="2:6">
       <c r="B40" s="3" t="s">
-        <v>373</v>
+        <v>367</v>
       </c>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
@@ -4505,24 +4487,24 @@
     </row>
     <row r="41" spans="2:6">
       <c r="B41" s="6" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
       <c r="C41" s="17" t="s">
-        <v>375</v>
+        <v>369</v>
       </c>
       <c r="D41" s="17" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="E41" s="17" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
     </row>
     <row r="42" spans="2:6">
       <c r="B42" s="4" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
       <c r="C42" s="18">
         <v>-2242535.295275593</v>
@@ -4534,12 +4516,12 @@
         <v>-1265194.807051147</v>
       </c>
       <c r="F42" s="26" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
     </row>
     <row r="43" spans="2:6">
       <c r="B43" s="4" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="C43" s="18">
         <v>-1870446.079396327</v>
@@ -4551,12 +4533,12 @@
         <v>-1094460.758228702</v>
       </c>
       <c r="F43" s="26" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
     </row>
     <row r="44" spans="2:6">
       <c r="B44" s="4" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="C44" s="18">
         <v>-1498356.863517062</v>
@@ -4568,7 +4550,7 @@
         <v>-923726.7094062574</v>
       </c>
       <c r="F44" s="26" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
     </row>
   </sheetData>
@@ -4598,7 +4580,7 @@
   <sheetData>
     <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -4607,12 +4589,12 @@
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="2" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
     </row>
     <row r="5" spans="2:6">
       <c r="B5" s="27" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="C5" s="27"/>
       <c r="D5" s="27"/>
@@ -4628,7 +4610,7 @@
     </row>
     <row r="9" spans="2:6">
       <c r="B9" s="3" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -4637,24 +4619,24 @@
     </row>
     <row r="10" spans="2:6">
       <c r="B10" s="6" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
     </row>
     <row r="11" spans="2:6">
       <c r="B11" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C11" s="18">
         <v>10000</v>
@@ -4669,7 +4651,7 @@
     </row>
     <row r="12" spans="2:6">
       <c r="B12" s="4" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="C12" s="18">
         <v>555000</v>
@@ -4684,7 +4666,7 @@
     </row>
     <row r="13" spans="2:6">
       <c r="B13" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="C13" s="18">
         <v>0</v>
@@ -4699,7 +4681,7 @@
     </row>
     <row r="14" spans="2:6">
       <c r="B14" s="4" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="C14" s="20">
         <v>-1870446.079396327</v>
@@ -4714,7 +4696,7 @@
     </row>
     <row r="15" spans="2:6">
       <c r="B15" s="4" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
       <c r="C15" s="20">
         <v>-557983.1555246152</v>
@@ -4729,7 +4711,7 @@
     </row>
     <row r="16" spans="2:6">
       <c r="B16" s="4" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
       <c r="C16" s="20">
         <v>-3762135.165624998</v>
@@ -4744,7 +4726,7 @@
     </row>
     <row r="18" spans="2:6">
       <c r="B18" s="3" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
@@ -4753,59 +4735,59 @@
     </row>
     <row r="19" spans="2:6">
       <c r="B19" s="4" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="C19" s="23">
         <v>1.121212121212121</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
     </row>
     <row r="20" spans="2:6">
       <c r="B20" s="4" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="C20" s="24">
         <v>0.8602001226515239</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
     </row>
     <row r="21" spans="2:6">
       <c r="B21" s="4" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="C21" s="23">
         <v>3.097257624777366</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
     </row>
     <row r="22" spans="2:6">
       <c r="B22" s="4" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="C22" s="20">
         <v>330000</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="E22" s="5"/>
       <c r="F22" s="5"/>
     </row>
     <row r="24" spans="2:6">
       <c r="B24" s="3" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
@@ -4814,7 +4796,7 @@
     </row>
     <row r="25" spans="2:6">
       <c r="B25" s="10" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
@@ -5318,7 +5300,7 @@
   <sheetPr>
     <tabColor rgb="FF1E3A5F"/>
   </sheetPr>
-  <dimension ref="B2:E22"/>
+  <dimension ref="B2:E19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="2.7109375" customWidth="1"/>
@@ -5369,182 +5351,156 @@
         <v>161</v>
       </c>
     </row>
-    <row r="7" spans="2:5">
-      <c r="B7" s="4" t="s">
+    <row r="8" spans="2:5">
+      <c r="B8" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+    </row>
+    <row r="9" spans="2:5">
+      <c r="B9" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" s="16">
+        <v>50000000</v>
+      </c>
+      <c r="D9" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="12" t="s">
+      <c r="E9" s="13" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="8" spans="2:5">
-      <c r="B8" s="4" t="s">
+    <row r="10" spans="2:5">
+      <c r="B10" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C10" s="16">
+        <v>10000000</v>
+      </c>
+      <c r="D10" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="12" t="s">
+      <c r="E10" s="12" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="11" spans="2:5">
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
     </row>
     <row r="12" spans="2:5">
       <c r="B12" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="C12" s="16">
-        <v>50000000</v>
-      </c>
-      <c r="D12" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="C12" s="5" t="s">
         <v>170</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="12" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="13" spans="2:5">
       <c r="B13" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="C13" s="16">
-        <v>10000000</v>
+      <c r="C13" s="14">
+        <v>180</v>
       </c>
       <c r="D13" s="12" t="s">
         <v>172</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="E13" s="13" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="14" spans="2:5">
-      <c r="B14" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="12" t="s">
+    <row r="15" spans="2:5">
+      <c r="B15" s="15" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="15" spans="2:5">
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+    </row>
+    <row r="16" spans="2:5">
+      <c r="B16" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C16" s="17" t="s">
         <v>176</v>
       </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="12" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="16" spans="2:5">
-      <c r="B16" s="4" t="s">
+      <c r="D16" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="C16" s="14">
+      <c r="E16" s="17" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5">
+      <c r="B17" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="C17" s="18">
+        <v>10000</v>
+      </c>
+      <c r="D17" s="18">
+        <v>555000</v>
+      </c>
+      <c r="E17" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5">
+      <c r="B18" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="D16" s="12" t="s">
-        <v>178</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="18" spans="2:5">
-      <c r="B18" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
+      <c r="C18" s="18">
+        <v>25000</v>
+      </c>
+      <c r="D18" s="18">
+        <v>376000</v>
+      </c>
+      <c r="E18" s="18">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" spans="2:5">
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C19" s="17" t="s">
-        <v>182</v>
-      </c>
-      <c r="D19" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="E19" s="17" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="20" spans="2:5">
-      <c r="B20" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="C20" s="18">
-        <v>10000</v>
-      </c>
-      <c r="D20" s="18">
-        <v>555000</v>
-      </c>
-      <c r="E20" s="18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="2:5">
-      <c r="B21" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="C21" s="18">
-        <v>25000</v>
-      </c>
-      <c r="D21" s="18">
-        <v>376000</v>
-      </c>
-      <c r="E21" s="18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="2:5">
-      <c r="B22" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="C22" s="18">
+      <c r="C19" s="18">
         <v>380000</v>
       </c>
-      <c r="D22" s="18">
+      <c r="D19" s="18">
         <v>225000</v>
       </c>
-      <c r="E22" s="18">
+      <c r="E19" s="18">
         <v>80000</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="5">
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="B15:E15"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E5" r:id="rId1"/>
-    <hyperlink ref="E12" r:id="rId2"/>
-    <hyperlink ref="E16" r:id="rId3"/>
+    <hyperlink ref="E9" r:id="rId2"/>
+    <hyperlink ref="E13" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5568,7 +5524,7 @@
   <sheetData>
     <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -5577,12 +5533,12 @@
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="2" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="2:6">
       <c r="B6" s="3" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -5594,16 +5550,16 @@
         <v>2</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" spans="2:6">
@@ -5611,13 +5567,13 @@
         <v>1</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="D8" s="16">
         <v>10000</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="F8" s="13" t="s">
         <v>42</v>
@@ -5626,7 +5582,7 @@
     <row r="9" spans="2:6">
       <c r="B9" s="5"/>
       <c r="C9" s="4" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="D9" s="19">
         <f>SUM(D8:D8)</f>
@@ -5637,7 +5593,7 @@
     </row>
     <row r="11" spans="2:6">
       <c r="B11" s="3" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -5649,16 +5605,16 @@
         <v>2</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="13" spans="2:6">
@@ -5666,13 +5622,13 @@
         <v>1</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="D13" s="16">
         <v>25000</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>47</v>
@@ -5681,7 +5637,7 @@
     <row r="14" spans="2:6">
       <c r="B14" s="5"/>
       <c r="C14" s="4" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="D14" s="19">
         <f>SUM(D13:D13)</f>
@@ -5692,7 +5648,7 @@
     </row>
     <row r="16" spans="2:6">
       <c r="B16" s="3" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
@@ -5704,16 +5660,16 @@
         <v>2</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="18" spans="2:6">
@@ -5721,13 +5677,13 @@
         <v>1</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="D18" s="16">
         <v>60000</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="F18" s="13" t="s">
         <v>72</v>
@@ -5738,13 +5694,13 @@
         <v>2</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="D19" s="16">
         <v>20000</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>67</v>
@@ -5755,13 +5711,13 @@
         <v>3</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="D20" s="16">
         <v>30000</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="F20" s="13" t="s">
         <v>67</v>
@@ -5772,13 +5728,13 @@
         <v>4</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="D21" s="16">
         <v>40000</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="F21" s="13" t="s">
         <v>42</v>
@@ -5789,13 +5745,13 @@
         <v>5</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="D22" s="16">
         <v>180000</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="F22" s="13" t="s">
         <v>82</v>
@@ -5806,13 +5762,13 @@
         <v>6</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="D23" s="16">
         <v>50000</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="F23" s="13" t="s">
         <v>92</v>
@@ -5821,7 +5777,7 @@
     <row r="24" spans="2:6">
       <c r="B24" s="5"/>
       <c r="C24" s="4" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="D24" s="19">
         <f>SUM(D18:D23)</f>
@@ -5869,7 +5825,7 @@
   <sheetData>
     <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -5878,12 +5834,12 @@
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="2" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="2:6">
       <c r="B6" s="3" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -5895,16 +5851,16 @@
         <v>2</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" spans="2:6">
@@ -5912,13 +5868,13 @@
         <v>1</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="D8" s="16">
         <v>390000</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="F8" s="13" t="s">
         <v>9</v>
@@ -5929,13 +5885,13 @@
         <v>2</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="D9" s="16">
         <v>75000</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="F9" s="13" t="s">
         <v>22</v>
@@ -5946,13 +5902,13 @@
         <v>3</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="D10" s="16">
         <v>50000</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="F10" s="13" t="s">
         <v>37</v>
@@ -5963,13 +5919,13 @@
         <v>4</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="D11" s="16">
         <v>40000</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="F11" s="13" t="s">
         <v>92</v>
@@ -5978,7 +5934,7 @@
     <row r="12" spans="2:6">
       <c r="B12" s="5"/>
       <c r="C12" s="4" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="D12" s="19">
         <f>SUM(D8:D11)</f>
@@ -5989,7 +5945,7 @@
     </row>
     <row r="14" spans="2:6">
       <c r="B14" s="3" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
@@ -6001,16 +5957,16 @@
         <v>2</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="16" spans="2:6">
@@ -6018,13 +5974,13 @@
         <v>1</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="D16" s="16">
         <v>180000</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="F16" s="13" t="s">
         <v>47</v>
@@ -6035,13 +5991,13 @@
         <v>2</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="D17" s="16">
         <v>36000</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="F17" s="13" t="s">
         <v>52</v>
@@ -6052,13 +6008,13 @@
         <v>3</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="D18" s="16">
         <v>130000</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="F18" s="13" t="s">
         <v>9</v>
@@ -6069,13 +6025,13 @@
         <v>4</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="D19" s="16">
         <v>20000</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>57</v>
@@ -6086,13 +6042,13 @@
         <v>5</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="D20" s="16">
         <v>10000</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="F20" s="13" t="s">
         <v>37</v>
@@ -6101,7 +6057,7 @@
     <row r="21" spans="2:6">
       <c r="B21" s="5"/>
       <c r="C21" s="4" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="D21" s="19">
         <f>SUM(D16:D20)</f>
@@ -6112,7 +6068,7 @@
     </row>
     <row r="23" spans="2:6">
       <c r="B23" s="3" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
@@ -6124,16 +6080,16 @@
         <v>2</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="25" spans="2:6">
@@ -6141,13 +6097,13 @@
         <v>1</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="D25" s="16">
         <v>145000</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>82</v>
@@ -6158,13 +6114,13 @@
         <v>2</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="D26" s="16">
         <v>30000</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="F26" s="13" t="s">
         <v>77</v>
@@ -6175,13 +6131,13 @@
         <v>3</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="D27" s="16">
         <v>25000</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="F27" s="13" t="s">
         <v>72</v>
@@ -6192,13 +6148,13 @@
         <v>4</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="D28" s="16">
         <v>15000</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="F28" s="13" t="s">
         <v>57</v>
@@ -6209,13 +6165,13 @@
         <v>5</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="D29" s="16">
         <v>10000</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="F29" s="13" t="s">
         <v>37</v>
@@ -6224,7 +6180,7 @@
     <row r="30" spans="2:6">
       <c r="B30" s="5"/>
       <c r="C30" s="4" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="D30" s="19">
         <f>SUM(D25:D29)</f>
@@ -6276,7 +6232,7 @@
   <sheetData>
     <row r="2" spans="2:10">
       <c r="B2" s="1" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -6288,35 +6244,35 @@
     </row>
     <row r="3" spans="2:10">
       <c r="B3" s="2" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5" spans="2:10">
       <c r="B5" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>242</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>246</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="6" spans="2:10">
       <c r="B6" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C6" s="18">
         <v>-10000</v>
@@ -6337,15 +6293,15 @@
         <v>0</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7" spans="2:10">
       <c r="B7" s="5" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="C7" s="18">
         <v>0</v>
@@ -6366,7 +6322,7 @@
         <v>-390000</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="J7" s="18">
         <v>-10000</v>
@@ -6374,7 +6330,7 @@
     </row>
     <row r="8" spans="2:10">
       <c r="B8" s="5" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="C8" s="18">
         <v>0</v>
@@ -6395,7 +6351,7 @@
         <v>-75000</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="J8" s="18">
         <v>-555000</v>
@@ -6403,7 +6359,7 @@
     </row>
     <row r="9" spans="2:10">
       <c r="B9" s="5" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="C9" s="18">
         <v>0</v>
@@ -6424,7 +6380,7 @@
         <v>-50000</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="J9" s="18">
         <v>0</v>
@@ -6432,7 +6388,7 @@
     </row>
     <row r="10" spans="2:10">
       <c r="B10" s="5" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="C10" s="18">
         <v>0</v>
@@ -6453,7 +6409,7 @@
         <v>-40000</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="J10" s="20">
         <f>H15</f>
@@ -6462,7 +6418,7 @@
     </row>
     <row r="11" spans="2:10">
       <c r="B11" s="4" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="C11" s="20">
         <f>SUM(C6:C10)</f>
@@ -6491,7 +6447,7 @@
     </row>
     <row r="12" spans="2:10">
       <c r="B12" s="5" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="C12" s="21">
         <f>1/(1+MARR)^0</f>
@@ -6520,7 +6476,7 @@
     </row>
     <row r="13" spans="2:10">
       <c r="B13" s="4" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="C13" s="20">
         <f>C11*C12</f>
@@ -6549,7 +6505,7 @@
     </row>
     <row r="14" spans="2:10">
       <c r="B14" s="4" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="C14" s="20">
         <f>C11</f>
@@ -6578,7 +6534,7 @@
     </row>
     <row r="15" spans="2:10">
       <c r="B15" s="4" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="C15" s="20">
         <f>C13</f>
@@ -6630,7 +6586,7 @@
   <sheetData>
     <row r="2" spans="2:10">
       <c r="B2" s="1" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -6642,35 +6598,35 @@
     </row>
     <row r="3" spans="2:10">
       <c r="B3" s="2" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" spans="2:10">
       <c r="B5" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>242</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>246</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="6" spans="2:10">
       <c r="B6" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C6" s="18">
         <v>-25000</v>
@@ -6691,15 +6647,15 @@
         <v>0</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7" spans="2:10">
       <c r="B7" s="5" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="C7" s="18">
         <v>0</v>
@@ -6720,7 +6676,7 @@
         <v>-180000</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="J7" s="18">
         <v>-25000</v>
@@ -6728,7 +6684,7 @@
     </row>
     <row r="8" spans="2:10">
       <c r="B8" s="5" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="C8" s="18">
         <v>0</v>
@@ -6749,7 +6705,7 @@
         <v>-36000</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="J8" s="18">
         <v>-376000</v>
@@ -6757,7 +6713,7 @@
     </row>
     <row r="9" spans="2:10">
       <c r="B9" s="5" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C9" s="18">
         <v>0</v>
@@ -6778,7 +6734,7 @@
         <v>-130000</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="J9" s="18">
         <v>0</v>
@@ -6786,7 +6742,7 @@
     </row>
     <row r="10" spans="2:10">
       <c r="B10" s="5" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C10" s="18">
         <v>0</v>
@@ -6807,7 +6763,7 @@
         <v>-20000</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="J10" s="20">
         <f>H16</f>
@@ -6816,7 +6772,7 @@
     </row>
     <row r="11" spans="2:10">
       <c r="B11" s="5" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C11" s="18">
         <v>0</v>
@@ -6839,7 +6795,7 @@
     </row>
     <row r="12" spans="2:10">
       <c r="B12" s="4" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="C12" s="20">
         <f>SUM(C6:C11)</f>
@@ -6868,7 +6824,7 @@
     </row>
     <row r="13" spans="2:10">
       <c r="B13" s="5" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="C13" s="21">
         <f>1/(1+MARR)^0</f>
@@ -6897,7 +6853,7 @@
     </row>
     <row r="14" spans="2:10">
       <c r="B14" s="4" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="C14" s="20">
         <f>C12*C13</f>
@@ -6926,7 +6882,7 @@
     </row>
     <row r="15" spans="2:10">
       <c r="B15" s="4" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="C15" s="20">
         <f>C12</f>
@@ -6955,7 +6911,7 @@
     </row>
     <row r="16" spans="2:10">
       <c r="B16" s="4" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="C16" s="20">
         <f>C14</f>
@@ -7007,7 +6963,7 @@
   <sheetData>
     <row r="2" spans="2:10">
       <c r="B2" s="1" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -7019,35 +6975,35 @@
     </row>
     <row r="3" spans="2:10">
       <c r="B3" s="2" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
     </row>
     <row r="5" spans="2:10">
       <c r="B5" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>242</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>246</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="6" spans="2:10">
       <c r="B6" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C6" s="18">
         <v>-380000</v>
@@ -7068,15 +7024,15 @@
         <v>0</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7" spans="2:10">
       <c r="B7" s="5" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="C7" s="18">
         <v>0</v>
@@ -7097,7 +7053,7 @@
         <v>-145000</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="J7" s="18">
         <v>-380000</v>
@@ -7105,7 +7061,7 @@
     </row>
     <row r="8" spans="2:10">
       <c r="B8" s="5" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="C8" s="18">
         <v>0</v>
@@ -7126,7 +7082,7 @@
         <v>-30000</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="J8" s="18">
         <v>-225000</v>
@@ -7134,7 +7090,7 @@
     </row>
     <row r="9" spans="2:10">
       <c r="B9" s="5" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="C9" s="18">
         <v>0</v>
@@ -7155,7 +7111,7 @@
         <v>-25000</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="J9" s="18">
         <v>80000</v>
@@ -7163,7 +7119,7 @@
     </row>
     <row r="10" spans="2:10">
       <c r="B10" s="5" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="C10" s="18">
         <v>0</v>
@@ -7184,7 +7140,7 @@
         <v>-15000</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="J10" s="22">
         <f>H17</f>
@@ -7193,7 +7149,7 @@
     </row>
     <row r="11" spans="2:10">
       <c r="B11" s="5" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C11" s="18">
         <v>0</v>
@@ -7216,7 +7172,7 @@
     </row>
     <row r="12" spans="2:10">
       <c r="B12" s="4" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="C12" s="18">
         <v>0</v>
@@ -7239,7 +7195,7 @@
     </row>
     <row r="13" spans="2:10">
       <c r="B13" s="4" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="C13" s="20">
         <f>SUM(C6:C12)</f>
@@ -7268,7 +7224,7 @@
     </row>
     <row r="14" spans="2:10">
       <c r="B14" s="5" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="C14" s="21">
         <f>1/(1+MARR)^0</f>
@@ -7297,7 +7253,7 @@
     </row>
     <row r="15" spans="2:10">
       <c r="B15" s="4" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="C15" s="20">
         <f>C13*C14</f>
@@ -7326,7 +7282,7 @@
     </row>
     <row r="16" spans="2:10">
       <c r="B16" s="4" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="C16" s="20">
         <f>C13</f>
@@ -7355,7 +7311,7 @@
     </row>
     <row r="17" spans="2:8">
       <c r="B17" s="4" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="C17" s="20">
         <f>C15</f>
@@ -7407,7 +7363,7 @@
   <sheetData>
     <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -7416,29 +7372,29 @@
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="2" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5" spans="2:6">
       <c r="B5" s="6" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6" spans="2:6">
       <c r="B6" s="4" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="C6" s="20">
         <f>'05. CF — Alt 1 Manual'!H15</f>
@@ -7453,12 +7409,12 @@
         <v>0</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
     </row>
     <row r="7" spans="2:6">
       <c r="B7" s="4" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="C7" s="20">
         <f>C6*MARR*(1+MARR)^STUDY_PERIOD/((1+MARR)^STUDY_PERIOD-1)</f>
@@ -7479,7 +7435,7 @@
     </row>
     <row r="8" spans="2:6">
       <c r="B8" s="4" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="C8" s="20">
         <f>C6*(1+MARR)^STUDY_PERIOD</f>
@@ -7500,7 +7456,7 @@
     </row>
     <row r="10" spans="2:6">
       <c r="B10" s="15" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="C10" s="15"/>
       <c r="D10" s="15"/>
@@ -7509,13 +7465,13 @@
     </row>
     <row r="11" spans="2:6">
       <c r="B11" s="5" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="C11" s="21">
         <v>3.352155098011401</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="E11" s="21">
         <v>0.4971767352982899</v>
@@ -7523,13 +7479,13 @@
     </row>
     <row r="12" spans="2:6">
       <c r="B12" s="5" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="C12" s="21">
         <v>0.2983155524615284</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="E12" s="21">
         <v>2.011357187499999</v>
@@ -7560,7 +7516,7 @@
   <sheetData>
     <row r="2" spans="2:9">
       <c r="B2" s="1" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -7571,12 +7527,12 @@
     </row>
     <row r="3" spans="2:9">
       <c r="B3" s="2" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" spans="2:9">
       <c r="B5" s="4" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="C5" s="20">
         <v>555000</v>
@@ -7584,7 +7540,7 @@
     </row>
     <row r="6" spans="2:9">
       <c r="B6" s="4" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C6" s="20">
         <v>10000</v>
@@ -7592,7 +7548,7 @@
     </row>
     <row r="9" spans="2:9">
       <c r="B9" s="3" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -7603,7 +7559,7 @@
     </row>
     <row r="10" spans="2:9">
       <c r="B10" s="4" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C10" s="20">
         <v>15000</v>
@@ -7611,7 +7567,7 @@
     </row>
     <row r="11" spans="2:9">
       <c r="B11" s="4" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C11" s="20">
         <v>179000</v>
@@ -7619,7 +7575,7 @@
     </row>
     <row r="12" spans="2:9">
       <c r="B12" s="5" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C12" s="18">
         <v>0</v>
@@ -7627,39 +7583,39 @@
     </row>
     <row r="13" spans="2:9">
       <c r="B13" s="4" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="C13" s="23">
         <f>C10/C11</f>
         <v>0</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
     </row>
     <row r="14" spans="2:9">
       <c r="B14" s="4" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
     </row>
     <row r="15" spans="2:9">
       <c r="B15" s="5" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="D15" s="18">
         <f>-C10</f>
@@ -7688,7 +7644,7 @@
     </row>
     <row r="16" spans="2:9">
       <c r="B16" s="4" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="D16" s="20">
         <f>D15</f>
@@ -7717,18 +7673,18 @@
     </row>
     <row r="17" spans="2:9">
       <c r="B17" s="4" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C17" s="23">
         <v>0.09636871508379888</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
     </row>
     <row r="19" spans="2:9">
       <c r="B19" s="3" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -7739,7 +7695,7 @@
     </row>
     <row r="20" spans="2:9">
       <c r="B20" s="4" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C20" s="20">
         <v>370000</v>
@@ -7747,7 +7703,7 @@
     </row>
     <row r="21" spans="2:9">
       <c r="B21" s="4" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C21" s="20">
         <v>330000</v>
@@ -7755,7 +7711,7 @@
     </row>
     <row r="22" spans="2:9">
       <c r="B22" s="5" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C22" s="18">
         <v>80000</v>
@@ -7763,39 +7719,39 @@
     </row>
     <row r="23" spans="2:9">
       <c r="B23" s="4" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="C23" s="23">
         <f>C20/C21</f>
         <v>0</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
     </row>
     <row r="24" spans="2:9">
       <c r="B24" s="4" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
     </row>
     <row r="25" spans="2:9">
       <c r="B25" s="5" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="D25" s="18">
         <f>-C20</f>
@@ -7824,7 +7780,7 @@
     </row>
     <row r="26" spans="2:9">
       <c r="B26" s="4" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="D26" s="20">
         <f>D25</f>
@@ -7853,18 +7809,18 @@
     </row>
     <row r="27" spans="2:9">
       <c r="B27" s="4" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C27" s="23">
         <v>1.33280303030303</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
     </row>
     <row r="30" spans="2:9">
       <c r="B30" s="15" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="C30" s="15"/>
       <c r="D30" s="15"/>
@@ -7875,7 +7831,7 @@
     </row>
     <row r="31" spans="2:9">
       <c r="B31" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="C31" s="7">
         <v>0</v>
@@ -7898,7 +7854,7 @@
     </row>
     <row r="32" spans="2:9">
       <c r="B32" s="4" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="C32" s="18">
         <v>-15000</v>
@@ -7921,7 +7877,7 @@
     </row>
     <row r="33" spans="2:8">
       <c r="B33" s="4" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="C33" s="18">
         <v>-370000</v>

</xml_diff>